<commit_message>
adding allen brain ontologies csv file
</commit_message>
<xml_diff>
--- a/apps/standardize_metadata.xlsx
+++ b/apps/standardize_metadata.xlsx
@@ -951,7 +951,7 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -962,6 +962,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00A933"/>
+        <bgColor rgb="FF008000"/>
       </patternFill>
     </fill>
   </fills>
@@ -999,12 +1005,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1021,6 +1035,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF00A933"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1048,7 +1122,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="13.5"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="0" t="s">
         <v>0</v>
       </c>
@@ -1070,10 +1144,10 @@
       <c r="H1" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="K1" s="0" t="s">
@@ -1097,7 +1171,7 @@
       <c r="Q1" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="3" t="s">
         <v>16</v>
       </c>
       <c r="S1" s="0" t="s">
@@ -1107,7 +1181,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="0" t="s">
         <v>19</v>
       </c>
@@ -1129,10 +1203,10 @@
       <c r="H2" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="J2" s="2" t="s">
         <v>27</v>
       </c>
       <c r="K2" s="0" t="s">
@@ -1157,7 +1231,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="0" t="s">
         <v>34</v>
       </c>
@@ -1167,6 +1241,8 @@
       <c r="H3" s="0" t="s">
         <v>36</v>
       </c>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
       <c r="K3" s="0" t="s">
         <v>37</v>
       </c>
@@ -1189,7 +1265,9 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
       <c r="M4" s="1" t="s">
         <v>43</v>
       </c>
@@ -1209,55 +1287,69 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
       <c r="O5" s="0" t="s">
         <v>48</v>
       </c>
       <c r="P5" s="0" t="s">
         <v>49</v>
       </c>
-      <c r="Q5" s="0" t="s">
+      <c r="Q5" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="R5" s="0" t="s">
+      <c r="R5" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
       <c r="O6" s="0" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
       <c r="O7" s="0" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
       <c r="O8" s="0" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
       <c r="O9" s="0" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
       <c r="O10" s="0" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
       <c r="Q11" s="0" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I12" s="0" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I12" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J12" s="0" t="s">
+      <c r="J12" s="2" t="s">
         <v>58</v>
       </c>
       <c r="K12" s="0" t="s">
@@ -1285,7 +1377,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
         <v>60</v>
       </c>
@@ -1307,10 +1399,10 @@
       <c r="H13" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I13" s="0" t="s">
+      <c r="I13" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="J13" s="0" t="s">
+      <c r="J13" s="2" t="s">
         <v>62</v>
       </c>
       <c r="K13" s="0" t="s">

</xml_diff>